<commit_message>
Align proposal narrative and reviewer path
</commit_message>
<xml_diff>
--- a/docs/Lead Applicant Scientific Milestones and Outcomes for Scaling AI Safety for a Multi-Agent World.xlsx
+++ b/docs/Lead Applicant Scientific Milestones and Outcomes for Scaling AI Safety for a Multi-Agent World.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Outcomes" sheetId="1" r:id="Ra234aec4dbe84916"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Outcomes" sheetId="1" r:id="R8b8d3bc501d044f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -143,7 +143,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -219,6 +219,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -482,16 +485,17 @@
         <x:v>Versioned campaign plans; machine-readable receipts; exact pooled interval and per-stratum diagnostics; measured paired SD and resulting descope decision; independent replay script; release tag.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="88" customHeight="1">
+    <x:row r="8" ht="84" hidden="0" customHeight="1">
       <x:c r="A8" s="24" t="str">
         <x:v>Q2 2027 (Month 6)</x:v>
       </x:c>
       <x:c r="B8" s="24" t="str">
-        <x:v>AN INTERPRETABLE POST-TRAINING AND TRANSFER TEST. Prompts, ordinary LoRA, and Progressive Denoising Distillation (PDD) face action-validity, rule-comprehension, impossible-regime, objective style, schema-preservation, same-game, and cross-game checks. The follower-rule classifier is validated against scripted labels and the tool-and-memory environment produces its first auditable traces.</x:v>
+        <x:v>AN INTERPRETABLE INTERVENTION CHANNEL - OR A SECOND DOCUMENTED FAILURE TO BUILD ONE. Prompts, ordinary LoRA, and Progressive Denoising Distillation (PDD) face action-validity, rule-comprehension, impossible-regime, objective style, schema-preservation, same-game, and cross-game checks. The follower-rule classifier is validated against scripted labels and the tool-and-memory environment produces its first auditable traces.</x:v>
       </x:c>
       <x:c r="C8" s="24" t="str">
-        <x:v>Frozen held-out set; per-model results and parse statistics; manifests and adapter hashes; same-game versus cross-game comparison including action diversity and synchronized collapse; classifier confusion matrix; tool/memory schema and first trace corpus.</x:v>
-      </x:c>
+        <x:v>Frozen held-out set; per-model results and parse statistics; manifests and adapter hashes; same-game versus cross-game comparison including action diversity and synchronized collapse; classifier confusion matrix; tool/memory schema and first trace corpus - or a failure report localizing the break in installation, schema, game performance, or transfer.</x:v>
+      </x:c>
+      <x:c r="D8" s="36"/>
     </x:row>
     <x:row r="9" ht="88" customHeight="1">
       <x:c r="A9" s="24" t="str">

</xml_diff>